<commit_message>
Implement initial version of CRN.parameter_map
</commit_message>
<xml_diff>
--- a/nanosuite/examples/edc_setup.xlsx
+++ b/nanosuite/examples/edc_setup.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="92">
   <si>
     <t xml:space="preserve">Parameters</t>
   </si>
@@ -168,34 +168,37 @@
     <t xml:space="preserve">Kidney</t>
   </si>
   <si>
+    <t xml:space="preserve">Probe 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spinal fluid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spleen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leaves</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fuel</t>
   </si>
   <si>
-    <t xml:space="preserve">Liver</t>
-  </si>
-  <si>
     <t xml:space="preserve">16_05_F</t>
   </si>
   <si>
-    <t xml:space="preserve">Heart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spinal fluid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spleen</t>
-  </si>
-  <si>
     <t xml:space="preserve">Input</t>
   </si>
   <si>
-    <t xml:space="preserve">Soil</t>
-  </si>
-  <si>
     <t xml:space="preserve">16_05_I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leaves</t>
   </si>
   <si>
     <t xml:space="preserve">Group</t>
@@ -661,7 +664,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AB18"/>
-  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38.7"/>
@@ -1279,8 +1282,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
-  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:R24"/>
+  <sheetFormatPr defaultColWidth="8.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.85"/>
@@ -1517,11 +1520,12 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21"/>
       <c r="B11" s="21" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D11" s="21" t="n">
         <v>1.5</v>
@@ -1530,122 +1534,195 @@
         <v>500</v>
       </c>
       <c r="F11" s="21" t="n">
-        <v>103</v>
+        <v>98.7</v>
       </c>
       <c r="G11" s="22" t="n">
         <f aca="false">(D11*E11)/F11</f>
-        <v>7.28155339805825</v>
+        <v>7.59878419452888</v>
       </c>
       <c r="J11" s="21"/>
       <c r="N11" s="21"/>
       <c r="Q11" s="0" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21" t="s">
-        <v>44</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21"/>
+      <c r="B12" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>500</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>92</v>
       </c>
       <c r="G12" s="22" t="n">
-        <v>484</v>
+        <f aca="false">(D12*E12)/F12</f>
+        <v>5.43478260869565</v>
       </c>
       <c r="H12" s="21"/>
       <c r="I12" s="21"/>
       <c r="Q12" s="0" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="22" t="n">
+        <f aca="false">E12-G12-G11</f>
+        <v>486.966433196776</v>
+      </c>
       <c r="H13" s="21"/>
       <c r="I13" s="21"/>
       <c r="N13" s="21"/>
       <c r="Q13" s="0" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21"/>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H14" s="21"/>
       <c r="I14" s="21"/>
       <c r="N14" s="21"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="F15" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="G15" s="21" t="s">
-        <v>31</v>
-      </c>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H15" s="21"/>
       <c r="I15" s="21"/>
       <c r="Q15" s="0" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="21" t="n">
-        <v>500</v>
-      </c>
-      <c r="F16" s="21" t="n">
-        <v>106</v>
-      </c>
-      <c r="G16" s="22" t="n">
-        <f aca="false">(D16*E16)/F16</f>
-        <v>4.71698113207547</v>
-      </c>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H16" s="21"/>
       <c r="I16" s="21"/>
       <c r="Q16" s="0" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>29</v>
+      </c>
       <c r="F17" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="G17" s="22" t="n">
-        <v>484</v>
+        <v>30</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>31</v>
       </c>
       <c r="H17" s="21"/>
       <c r="I17" s="21"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>500</v>
+      </c>
+      <c r="F18" s="21" t="n">
+        <v>103</v>
+      </c>
+      <c r="G18" s="22" t="n">
+        <f aca="false">(D18*E18)/F18</f>
+        <v>7.28155339805825</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="21"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="21"/>
       <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
+      <c r="D22" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>31</v>
+      </c>
       <c r="H22" s="21"/>
       <c r="I22" s="21"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21"/>
+      <c r="B23" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>500</v>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>106</v>
+      </c>
+      <c r="G23" s="22" t="n">
+        <f aca="false">(D23*E23)/F23</f>
+        <v>4.71698113207547</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="G24" s="22" t="n">
+        <v>484</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1670,7 +1747,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N37"/>
-  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5859375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="11.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.43"/>
@@ -1689,54 +1766,54 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="25" t="s">
         <v>24</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E1" s="25" t="s">
         <v>23</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G1" s="25" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H1" s="25" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J1" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K1" s="25" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L1" s="25" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M1" s="25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N1" s="25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C2" s="21" t="s">
         <v>26</v>
@@ -1752,7 +1829,7 @@
         <v>100</v>
       </c>
       <c r="G2" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H2" s="21" t="n">
         <v>0</v>
@@ -1764,13 +1841,13 @@
         <v>10</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L2" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N2" s="23" t="n">
         <v>0</v>
@@ -1779,7 +1856,7 @@
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="26"/>
       <c r="B3" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>26</v>
@@ -1795,7 +1872,7 @@
         <v>100</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H3" s="21" t="n">
         <v>0</v>
@@ -1807,13 +1884,13 @@
         <v>10</v>
       </c>
       <c r="K3" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L3" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M3" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N3" s="23" t="n">
         <v>0</v>
@@ -1822,7 +1899,7 @@
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="26"/>
       <c r="B4" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" s="21" t="s">
         <v>26</v>
@@ -1838,7 +1915,7 @@
         <v>100</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H4" s="21" t="n">
         <v>0</v>
@@ -1850,13 +1927,13 @@
         <v>10</v>
       </c>
       <c r="K4" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L4" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M4" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N4" s="23" t="n">
         <v>0</v>
@@ -1865,7 +1942,7 @@
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26"/>
       <c r="B5" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C5" s="21" t="s">
         <v>26</v>
@@ -1881,7 +1958,7 @@
         <v>100</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>5</v>
@@ -1893,13 +1970,13 @@
         <v>10</v>
       </c>
       <c r="K5" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L5" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M5" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N5" s="23" t="n">
         <v>0</v>
@@ -1908,7 +1985,7 @@
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26"/>
       <c r="B6" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>26</v>
@@ -1920,28 +1997,28 @@
         <v>25</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>10</v>
       </c>
       <c r="I6" s="21" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="J6" s="21" t="n">
         <v>10</v>
       </c>
       <c r="K6" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L6" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M6" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N6" s="23" t="n">
         <v>0</v>
@@ -1950,7 +2027,7 @@
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26"/>
       <c r="B7" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="21" t="s">
         <v>26</v>
@@ -1962,28 +2039,28 @@
         <v>25</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H7" s="21" t="n">
         <v>50</v>
       </c>
       <c r="I7" s="21" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="J7" s="21" t="n">
         <v>10</v>
       </c>
       <c r="K7" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L7" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M7" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N7" s="23" t="n">
         <v>0</v>
@@ -1992,7 +2069,7 @@
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26"/>
       <c r="B8" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>26</v>
@@ -2008,25 +2085,25 @@
         <v>100</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>100</v>
       </c>
       <c r="I8" s="21" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="J8" s="21" t="n">
         <v>10</v>
       </c>
       <c r="K8" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L8" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M8" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N8" s="23" t="n">
         <v>0</v>
@@ -2035,7 +2112,7 @@
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26"/>
       <c r="B9" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C9" s="21" t="s">
         <v>26</v>
@@ -2051,25 +2128,25 @@
         <v>100</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>500</v>
       </c>
       <c r="I9" s="21" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="J9" s="21" t="n">
         <v>10</v>
       </c>
       <c r="K9" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L9" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M9" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N9" s="23" t="n">
         <v>0</v>
@@ -2078,7 +2155,7 @@
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26"/>
       <c r="B10" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C10" s="21" t="s">
         <v>26</v>
@@ -2094,25 +2171,25 @@
         <v>100</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="I10" s="21" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="J10" s="21" t="n">
         <v>10</v>
       </c>
       <c r="K10" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L10" s="21" t="n">
         <v>15</v>
       </c>
       <c r="M10" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N10" s="23" t="n">
         <v>0</v>
@@ -2120,10 +2197,10 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C11" s="21" t="s">
         <v>26</v>
@@ -2139,7 +2216,7 @@
         <v>100</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H11" s="21" t="n">
         <v>0</v>
@@ -2151,13 +2228,13 @@
         <v>0</v>
       </c>
       <c r="K11" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="M11" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N11" s="23" t="n">
         <v>0</v>
@@ -2166,7 +2243,7 @@
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26"/>
       <c r="B12" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C12" s="21" t="s">
         <v>26</v>
@@ -2182,7 +2259,7 @@
         <v>100</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H12" s="21" t="n">
         <v>0</v>
@@ -2194,13 +2271,13 @@
         <v>10</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L12" s="21" t="n">
         <v>0</v>
       </c>
       <c r="M12" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N12" s="23" t="n">
         <v>0</v>
@@ -2208,10 +2285,10 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C13" s="21" t="s">
         <v>26</v>
@@ -2227,7 +2304,7 @@
         <v>100</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H13" s="21" t="n">
         <v>0</v>
@@ -2239,13 +2316,13 @@
         <v>10</v>
       </c>
       <c r="K13" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L13" s="21" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N13" s="23" t="n">
         <v>0</v>
@@ -2254,7 +2331,7 @@
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26"/>
       <c r="B14" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C14" s="21" t="s">
         <v>26</v>
@@ -2270,7 +2347,7 @@
         <v>100</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>0</v>
@@ -2282,13 +2359,13 @@
         <v>8</v>
       </c>
       <c r="K14" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L14" s="21" t="n">
         <v>13</v>
       </c>
       <c r="M14" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N14" s="23" t="n">
         <v>2</v>
@@ -2297,7 +2374,7 @@
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="26"/>
       <c r="B15" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C15" s="21" t="s">
         <v>26</v>
@@ -2313,7 +2390,7 @@
         <v>100</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H15" s="21" t="n">
         <v>0</v>
@@ -2325,13 +2402,13 @@
         <v>6</v>
       </c>
       <c r="K15" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L15" s="21" t="n">
         <v>11</v>
       </c>
       <c r="M15" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N15" s="23" t="n">
         <v>4</v>
@@ -2340,7 +2417,7 @@
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26"/>
       <c r="B16" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C16" s="21" t="s">
         <v>26</v>
@@ -2356,7 +2433,7 @@
         <v>100</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H16" s="21" t="n">
         <v>0</v>
@@ -2368,13 +2445,13 @@
         <v>4</v>
       </c>
       <c r="K16" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L16" s="21" t="n">
         <v>9</v>
       </c>
       <c r="M16" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N16" s="23" t="n">
         <v>6</v>
@@ -2383,7 +2460,7 @@
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26"/>
       <c r="B17" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C17" s="21" t="s">
         <v>26</v>
@@ -2399,7 +2476,7 @@
         <v>100</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H17" s="21" t="n">
         <v>0</v>
@@ -2411,13 +2488,13 @@
         <v>2</v>
       </c>
       <c r="K17" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L17" s="21" t="n">
         <v>7</v>
       </c>
       <c r="M17" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N17" s="23" t="n">
         <v>8</v>
@@ -2425,10 +2502,10 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C18" s="21" t="s">
         <v>26</v>
@@ -2444,7 +2521,7 @@
         <v>100</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H18" s="21" t="n">
         <v>0</v>
@@ -2456,13 +2533,13 @@
         <v>0</v>
       </c>
       <c r="K18" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L18" s="21" t="n">
         <v>5</v>
       </c>
       <c r="M18" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N18" s="23" t="n">
         <v>10</v>
@@ -2471,7 +2548,7 @@
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26"/>
       <c r="B19" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C19" s="21" t="s">
         <v>26</v>
@@ -2487,7 +2564,7 @@
         <v>100</v>
       </c>
       <c r="G19" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H19" s="21" t="n">
         <v>0</v>
@@ -2499,13 +2576,13 @@
         <v>0</v>
       </c>
       <c r="K19" s="21" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L19" s="21" t="n">
         <v>5</v>
       </c>
       <c r="M19" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N19" s="23" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Read controls from setup file
Samples now have associated controls given by the "Positive"
and "Negative" columns in the setup file. These are stored
along the content coordinate as Assay.setup.positive and
Assay.setup.negative.
</commit_message>
<xml_diff>
--- a/nanosuite/examples/edc_setup.xlsx
+++ b/nanosuite/examples/edc_setup.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="92">
   <si>
     <t xml:space="preserve">Parameters</t>
   </si>
@@ -207,6 +207,12 @@
     <t xml:space="preserve">Sample ID</t>
   </si>
   <si>
+    <t xml:space="preserve">Negative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positive</t>
+  </si>
+  <si>
     <t xml:space="preserve">Media % assay</t>
   </si>
   <si>
@@ -264,9 +270,6 @@
     <t xml:space="preserve">Sample X9</t>
   </si>
   <si>
-    <t xml:space="preserve">Negative</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sample X10</t>
   </si>
   <si>
@@ -289,9 +292,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sample X16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Positive</t>
   </si>
   <si>
     <t xml:space="preserve">Sample X17</t>
@@ -1230,46 +1230,46 @@
     <mergeCell ref="A13:B13"/>
   </mergeCells>
   <dataValidations count="9">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F11" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F11" type="list">
       <formula1>"Clariostar 1,Clariostar 2,Clariostar 3,Clariostar 4,Clariostar 5"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B4" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B4" type="whole">
       <formula1>10</formula1>
       <formula2>50</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B5" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B5" type="whole">
       <formula1>1000</formula1>
       <formula2>3000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B10" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B10" type="list">
       <formula1>"Alex (AWJ),Jasmine (JB),Maria (MO),Ennio (EL),Cheryl (CA),Tarin (TT),Esther (EM),Hyeyun (HJ)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B7" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B7" type="list">
       <formula1>"Greiner 348 hibase (784900),Greiner 96 (655900)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B8" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B8" type="whole">
       <formula1>3</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B9" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B9" type="list">
       <formula1>"Alex (AWJ),Jasmine (JEB),Maria (MO),Ennio (EL),Cheryl (CA),Tarin (TT),Esther (EM),Hyeyun (HJ)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B3" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B3" type="list">
       <formula1>"Clariostar 1,Clariostar 2,Clariostar 3,Clariostar 4,Clariostar 5,Unkonwn"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B6" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B6" type="whole">
       <formula1>5</formula1>
       <formula2>15</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1726,14 +1726,14 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="Q2:Q1016" type="none">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="Q2:Q1016" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1746,22 +1746,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultColWidth="8.5859375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="23" width="11.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="23" width="17.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="23" width="11.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="23" width="17.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1772,776 +1772,782 @@
         <v>60</v>
       </c>
       <c r="C1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="25" t="s">
+      <c r="F1" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="G1" s="25" t="s">
+      <c r="H1" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="25" t="s">
         <v>57</v>
-      </c>
-      <c r="H1" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="I1" s="25" t="s">
-        <v>64</v>
       </c>
       <c r="J1" s="25" t="s">
         <v>65</v>
       </c>
       <c r="K1" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="L1" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="M1" s="25" t="s">
         <v>55</v>
-      </c>
-      <c r="L1" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="M1" s="25" t="s">
-        <v>67</v>
       </c>
       <c r="N1" s="25" t="s">
         <v>68</v>
       </c>
+      <c r="O1" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="P1" s="25" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="21" t="n">
+        <f aca="false">100-F2</f>
+        <v>100</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="J2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="M2" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="N2" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="O2" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="21" t="n">
-        <f aca="false">100-D2</f>
-        <v>100</v>
-      </c>
-      <c r="G2" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="H2" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="K2" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="L2" s="21" t="n">
-        <v>15</v>
-      </c>
-      <c r="M2" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N2" s="23" t="n">
+      <c r="P2" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="26"/>
       <c r="B3" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="21" t="s">
+      <c r="F3" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="21" t="n">
-        <f aca="false">100-D3</f>
+      <c r="H3" s="21" t="n">
+        <f aca="false">100-F3</f>
         <v>100</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="I3" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="21" t="s">
+      <c r="J3" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="21" t="n">
+      <c r="L3" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K3" s="21" t="s">
+      <c r="M3" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L3" s="21" t="n">
+      <c r="N3" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="M3" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N3" s="23" t="n">
+      <c r="O3" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P3" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="26"/>
       <c r="B4" s="0" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="21" t="s">
+      <c r="F4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="21" t="n">
-        <f aca="false">100-D4</f>
+      <c r="H4" s="21" t="n">
+        <f aca="false">100-F4</f>
         <v>100</v>
       </c>
-      <c r="G4" s="21" t="s">
+      <c r="I4" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H4" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="21" t="s">
+      <c r="J4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="21" t="n">
+      <c r="L4" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K4" s="21" t="s">
+      <c r="M4" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L4" s="21" t="n">
+      <c r="N4" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="M4" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N4" s="23" t="n">
+      <c r="O4" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P4" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26"/>
       <c r="B5" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="21" t="s">
+      <c r="F5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="21" t="n">
-        <f aca="false">100-D5</f>
+      <c r="H5" s="21" t="n">
+        <f aca="false">100-F5</f>
         <v>100</v>
       </c>
-      <c r="G5" s="21" t="s">
+      <c r="I5" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H5" s="21" t="n">
+      <c r="J5" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="I5" s="21" t="s">
+      <c r="K5" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="21" t="n">
+      <c r="L5" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K5" s="21" t="s">
+      <c r="M5" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L5" s="21" t="n">
+      <c r="N5" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="M5" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N5" s="23" t="n">
+      <c r="O5" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P5" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26"/>
       <c r="B6" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="21" t="s">
+      <c r="F6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="G6" s="21" t="s">
+      <c r="H6" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="I6" s="21" t="s">
         <v>57</v>
-      </c>
-      <c r="H6" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="I6" s="21" t="s">
-        <v>48</v>
       </c>
       <c r="J6" s="21" t="n">
         <v>10</v>
       </c>
       <c r="K6" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L6" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="M6" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L6" s="21" t="n">
+      <c r="N6" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="M6" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N6" s="23" t="n">
+      <c r="O6" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P6" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26"/>
       <c r="B7" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="21" t="s">
+      <c r="F7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="G7" s="21" t="s">
+      <c r="H7" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="I7" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="J7" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="K7" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="L7" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K7" s="21" t="s">
+      <c r="M7" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L7" s="21" t="n">
+      <c r="N7" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="M7" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N7" s="23" t="n">
+      <c r="O7" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P7" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26"/>
       <c r="B8" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="21" t="s">
+      <c r="F8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="21" t="n">
-        <f aca="false">100-D8</f>
+      <c r="H8" s="21" t="n">
+        <f aca="false">100-F8</f>
         <v>100</v>
       </c>
-      <c r="G8" s="21" t="s">
+      <c r="I8" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="J8" s="21" t="n">
         <v>100</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="K8" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="J8" s="21" t="n">
+      <c r="L8" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K8" s="21" t="s">
+      <c r="M8" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L8" s="21" t="n">
+      <c r="N8" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="M8" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N8" s="23" t="n">
+      <c r="O8" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P8" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26"/>
       <c r="B9" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="21" t="s">
+      <c r="F9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="21" t="n">
-        <f aca="false">100-D9</f>
+      <c r="H9" s="21" t="n">
+        <f aca="false">100-F9</f>
         <v>100</v>
       </c>
-      <c r="G9" s="21" t="s">
+      <c r="I9" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="21" t="n">
+      <c r="J9" s="21" t="n">
         <v>500</v>
       </c>
-      <c r="I9" s="21" t="s">
+      <c r="K9" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="J9" s="21" t="n">
+      <c r="L9" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K9" s="21" t="s">
+      <c r="M9" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L9" s="21" t="n">
+      <c r="N9" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="M9" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N9" s="23" t="n">
+      <c r="O9" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P9" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26"/>
       <c r="B10" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="C10" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="E10" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="21" t="s">
+      <c r="F10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="21" t="n">
-        <f aca="false">100-D10</f>
+      <c r="H10" s="21" t="n">
+        <f aca="false">100-F10</f>
         <v>100</v>
       </c>
-      <c r="G10" s="21" t="s">
+      <c r="I10" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H10" s="21" t="n">
+      <c r="J10" s="21" t="n">
         <v>1000</v>
       </c>
-      <c r="I10" s="21" t="s">
+      <c r="K10" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="21" t="n">
+      <c r="L10" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K10" s="21" t="s">
+      <c r="M10" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L10" s="21" t="n">
+      <c r="N10" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="M10" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N10" s="23" t="n">
+      <c r="O10" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P10" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E11" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="21" t="s">
+      <c r="F11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="21" t="n">
-        <f aca="false">100-D11</f>
+      <c r="H11" s="21" t="n">
+        <f aca="false">100-F11</f>
         <v>100</v>
       </c>
-      <c r="G11" s="21" t="s">
+      <c r="I11" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="21" t="s">
+      <c r="J11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="21" t="s">
+      <c r="L11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N11" s="23" t="n">
+      <c r="N11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P11" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26"/>
       <c r="B12" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="21" t="s">
+      <c r="F12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="21" t="n">
-        <f aca="false">100-D12</f>
+      <c r="H12" s="21" t="n">
+        <f aca="false">100-F12</f>
         <v>100</v>
       </c>
-      <c r="G12" s="21" t="s">
+      <c r="I12" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="21" t="s">
+      <c r="J12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J12" s="21" t="n">
+      <c r="L12" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K12" s="21" t="s">
+      <c r="M12" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N12" s="23" t="n">
+      <c r="N12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P12" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="21" t="s">
+      <c r="F13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="21" t="n">
-        <f aca="false">100-D13</f>
+      <c r="H13" s="21" t="n">
+        <f aca="false">100-F13</f>
         <v>100</v>
       </c>
-      <c r="G13" s="21" t="s">
+      <c r="I13" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="21" t="s">
+      <c r="J13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J13" s="21" t="n">
+      <c r="L13" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="K13" s="21" t="s">
+      <c r="M13" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N13" s="23" t="n">
+      <c r="N13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P13" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26"/>
       <c r="B14" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="C14" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="E14" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="21" t="s">
+      <c r="F14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="21" t="n">
-        <f aca="false">100-D14</f>
+      <c r="H14" s="21" t="n">
+        <f aca="false">100-F14</f>
         <v>100</v>
       </c>
-      <c r="G14" s="21" t="s">
+      <c r="I14" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="21" t="s">
+      <c r="J14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J14" s="21" t="n">
+      <c r="L14" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="K14" s="21" t="s">
+      <c r="M14" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L14" s="21" t="n">
+      <c r="N14" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="M14" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N14" s="23" t="n">
+      <c r="O14" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P14" s="23" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="26"/>
       <c r="B15" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="21" t="s">
+      <c r="F15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="21" t="n">
-        <f aca="false">100-D15</f>
+      <c r="H15" s="21" t="n">
+        <f aca="false">100-F15</f>
         <v>100</v>
       </c>
-      <c r="G15" s="21" t="s">
+      <c r="I15" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="21" t="s">
+      <c r="J15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J15" s="21" t="n">
+      <c r="L15" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="K15" s="21" t="s">
+      <c r="M15" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L15" s="21" t="n">
+      <c r="N15" s="21" t="n">
         <v>11</v>
       </c>
-      <c r="M15" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N15" s="23" t="n">
+      <c r="O15" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P15" s="23" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26"/>
       <c r="B16" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="C16" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="21" t="s">
+      <c r="F16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="21" t="n">
-        <f aca="false">100-D16</f>
+      <c r="H16" s="21" t="n">
+        <f aca="false">100-F16</f>
         <v>100</v>
       </c>
-      <c r="G16" s="21" t="s">
+      <c r="I16" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="21" t="s">
+      <c r="J16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J16" s="21" t="n">
+      <c r="L16" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K16" s="21" t="s">
+      <c r="M16" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L16" s="21" t="n">
+      <c r="N16" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="M16" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N16" s="23" t="n">
+      <c r="O16" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P16" s="23" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26"/>
       <c r="B17" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="E17" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="21" t="s">
+      <c r="F17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F17" s="21" t="n">
-        <f aca="false">100-D17</f>
+      <c r="H17" s="21" t="n">
+        <f aca="false">100-F17</f>
         <v>100</v>
       </c>
-      <c r="G17" s="21" t="s">
+      <c r="I17" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="21" t="s">
+      <c r="J17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J17" s="21" t="n">
+      <c r="L17" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K17" s="21" t="s">
+      <c r="M17" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L17" s="21" t="n">
+      <c r="N17" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="M17" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N17" s="23" t="n">
+      <c r="O17" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P17" s="23" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>89</v>
+        <v>62</v>
       </c>
       <c r="B18" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="E18" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="21" t="s">
+      <c r="F18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F18" s="21" t="n">
-        <f aca="false">100-D18</f>
+      <c r="H18" s="21" t="n">
+        <f aca="false">100-F18</f>
         <v>100</v>
       </c>
-      <c r="G18" s="21" t="s">
+      <c r="I18" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="21" t="s">
+      <c r="J18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="21" t="s">
+      <c r="L18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L18" s="21" t="n">
+      <c r="N18" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="M18" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N18" s="23" t="n">
+      <c r="O18" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P18" s="23" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2550,47 +2556,45 @@
       <c r="B19" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="E19" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="21" t="s">
+      <c r="F19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F19" s="21" t="n">
-        <f aca="false">100-D19</f>
+      <c r="H19" s="21" t="n">
+        <f aca="false">100-F19</f>
         <v>100</v>
       </c>
-      <c r="G19" s="21" t="s">
+      <c r="I19" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="H19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="21" t="s">
+      <c r="J19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="J19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="21" t="s">
+      <c r="L19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L19" s="21" t="n">
+      <c r="N19" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="M19" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="N19" s="23" t="n">
+      <c r="O19" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P19" s="23" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
       <c r="E20" s="21"/>
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
@@ -2599,10 +2603,10 @@
       <c r="J20" s="21"/>
       <c r="K20" s="21"/>
       <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
@@ -2611,10 +2615,10 @@
       <c r="J21" s="21"/>
       <c r="K21" s="21"/>
       <c r="L21" s="21"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="21"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
       <c r="E22" s="21"/>
       <c r="F22" s="21"/>
       <c r="G22" s="21"/>
@@ -2623,10 +2627,10 @@
       <c r="J22" s="21"/>
       <c r="K22" s="21"/>
       <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
       <c r="E23" s="21"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
@@ -2635,10 +2639,10 @@
       <c r="J23" s="21"/>
       <c r="K23" s="21"/>
       <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
       <c r="E24" s="21"/>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
@@ -2647,10 +2651,10 @@
       <c r="J24" s="21"/>
       <c r="K24" s="21"/>
       <c r="L24" s="21"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="21"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
       <c r="E25" s="21"/>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
@@ -2659,10 +2663,10 @@
       <c r="J25" s="21"/>
       <c r="K25" s="21"/>
       <c r="L25" s="21"/>
+      <c r="M25" s="21"/>
+      <c r="N25" s="21"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
       <c r="E26" s="21"/>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
@@ -2671,10 +2675,10 @@
       <c r="J26" s="21"/>
       <c r="K26" s="21"/>
       <c r="L26" s="21"/>
+      <c r="M26" s="21"/>
+      <c r="N26" s="21"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
       <c r="E27" s="21"/>
       <c r="F27" s="21"/>
       <c r="G27" s="21"/>
@@ -2683,10 +2687,10 @@
       <c r="J27" s="21"/>
       <c r="K27" s="21"/>
       <c r="L27" s="21"/>
+      <c r="M27" s="21"/>
+      <c r="N27" s="21"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
       <c r="E28" s="21"/>
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
@@ -2695,10 +2699,10 @@
       <c r="J28" s="21"/>
       <c r="K28" s="21"/>
       <c r="L28" s="21"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="21"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
       <c r="E29" s="21"/>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
@@ -2707,10 +2711,10 @@
       <c r="J29" s="21"/>
       <c r="K29" s="21"/>
       <c r="L29" s="21"/>
+      <c r="M29" s="21"/>
+      <c r="N29" s="21"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
       <c r="E30" s="21"/>
       <c r="F30" s="21"/>
       <c r="G30" s="21"/>
@@ -2719,10 +2723,10 @@
       <c r="J30" s="21"/>
       <c r="K30" s="21"/>
       <c r="L30" s="21"/>
+      <c r="M30" s="21"/>
+      <c r="N30" s="21"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
       <c r="E31" s="21"/>
       <c r="F31" s="21"/>
       <c r="G31" s="21"/>
@@ -2731,10 +2735,10 @@
       <c r="J31" s="21"/>
       <c r="K31" s="21"/>
       <c r="L31" s="21"/>
+      <c r="M31" s="21"/>
+      <c r="N31" s="21"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
       <c r="E32" s="21"/>
       <c r="F32" s="21"/>
       <c r="G32" s="21"/>
@@ -2743,10 +2747,10 @@
       <c r="J32" s="21"/>
       <c r="K32" s="21"/>
       <c r="L32" s="21"/>
+      <c r="M32" s="21"/>
+      <c r="N32" s="21"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
       <c r="E33" s="21"/>
       <c r="F33" s="21"/>
       <c r="G33" s="21"/>
@@ -2755,22 +2759,24 @@
       <c r="J33" s="21"/>
       <c r="K33" s="21"/>
       <c r="L33" s="21"/>
+      <c r="M33" s="21"/>
+      <c r="N33" s="21"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I34" s="21"/>
-      <c r="J34" s="21"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I35" s="21"/>
-      <c r="J35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I36" s="21"/>
-      <c r="J36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I37" s="21"/>
-      <c r="J37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2780,30 +2786,30 @@
     <mergeCell ref="A18:A19"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I2:I1019" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="K2:K1019" type="list">
       <formula1>stock_solutions!$A$3:$A$23</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C1019" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E2:E1019" type="list">
       <formula1>stock_solutions!$Q$3:$Q$400</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="K2:K1019" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="M2:M1019" type="list">
       <formula1>stock_solutions!$A$3:$A$1048576</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E2:E1019" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G1019" type="list">
       <formula1>stock_solutions!$L$2:$L$1048576</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G168" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I2:I168" type="list">
       <formula1>stock_solutions!$A$2:$A$166</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>